<commit_message>
feat: dashboard interativo com filtros e JSON externo
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_gerencial_padronizado.xlsx
+++ b/relatorios/relatorio_gerencial_padronizado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,16 +467,16 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46054</v>
+        <v>46030</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Venda projeto A</t>
+          <t>Mensalidade carteira premium</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>15000</v>
+        <v>8400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -494,61 +494,61 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>15000</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46056</v>
+        <v>46034</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pagamento fornecedor X</t>
+          <t>Projeto de implantacao alfa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4200.5</v>
+        <v>12600</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>consultoria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-4200.5</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46063</v>
+        <v>46037</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Assinatura software</t>
+          <t>Midia de aquisicao</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -557,65 +557,65 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>899.9</v>
+        <v>1850.45</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-899.9</v>
+        <v>-1850.45</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46068</v>
+        <v>46042</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Venda projeto B</t>
+          <t>Infraestrutura em nuvem</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>8700</v>
+        <v>920.3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>comercial</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>8700</v>
+        <v>-920.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46086</v>
+        <v>46050</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Folha salarial</t>
+          <t>Folha operacional</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -629,34 +629,34 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>6800</v>
+        <v>5400</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>rh</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>-6800</v>
+        <v>-5400</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46095</v>
+        <v>46058</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Recebimento consultoria</t>
+          <t>Renovacao contratos B2B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -665,56 +665,1244 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4600</v>
+        <v>9100</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>consultoria</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4600</v>
+        <v>9100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46101</v>
+        <v>46062</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Energia eletrica</t>
+          <t>Treinamento corporativo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fornecedor homologado</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>4100.8</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>-4100.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ferramentas analiticas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1180.25</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>-1180.25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Comissao comercial</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2890</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>-2890</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Projeto de integracao beta</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>14850</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>14850</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Receita de suporte premium</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>4650</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>sucesso_cliente</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>4650</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Campanha de retencao</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2310.1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>-2310.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Licencas de software</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1340.6</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>-1340.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Folha salarial</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>6120</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>-6120</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pacote de consultoria recorrente</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>6900</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Expansao de contas enterprise</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>vendas</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>11800</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>11800</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Viagens comerciais</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1740.55</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>-1740.55</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Servicos terceirizados</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4525</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>-4525</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Energia e utilidades</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>infraestrutura</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>despesa</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>740.3099999999999</v>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>860.9</v>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>adm</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>-740.3099999999999</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>-860.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Novos contratos SMB</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>vendas</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>9700</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Receita de onboarding</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4300</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Eventos e comunidade</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2088.4</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>-2088.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Upgrade de seguranca</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>980.15</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>-980.15</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Beneficios e encargos</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>6335.2</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>-6335.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Projeto analytics gamma</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>16300</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>16300</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Receita de renovacao anual</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>8800</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>8800</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Parceiros estrategicos</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>3895</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>-3895</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Monitoramento de plataforma</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1125.8</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>-1125.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Aluguel escritorio</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2790</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>-2790</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Squad dedicado delta</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>17150</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>17150</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pacote de suporte enterprise</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>5400</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>sucesso_cliente</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Recrutamento especializado</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>6840</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>-6840</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Campanha ABM</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>2645.7</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>-2645.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Automacao de backoffice</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1495.35</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>-1495.35</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Renovacao base enterprise</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>10200</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Projeto de performance epsilon</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>15400</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Operacao de campo</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1985.25</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>-1985.25</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Compliance e auditoria</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>-1320</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Folha variavel e bonus</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>7210</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>-7210</v>
       </c>
     </row>
   </sheetData>
@@ -728,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,33 +1944,129 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5100.4</v>
+        <v>8170.75</v>
       </c>
       <c r="C2" t="n">
-        <v>23700</v>
+        <v>21000</v>
       </c>
       <c r="D2" t="n">
-        <v>18599.6</v>
+        <v>12829.25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8171.05</v>
+      </c>
+      <c r="C3" t="n">
+        <v>14300</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6128.95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>7540.309999999999</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4600</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-2940.309999999999</v>
+      <c r="B4" t="n">
+        <v>9770.700000000001</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>9729.299999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7126.45</v>
+      </c>
+      <c r="C5" t="n">
+        <v>18700</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11573.55</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9403.75</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4596.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7810.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="D7" t="n">
+        <v>17289.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>10981.05</v>
+      </c>
+      <c r="C8" t="n">
+        <v>22550</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11568.95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10515.25</v>
+      </c>
+      <c r="C9" t="n">
+        <v>25600</v>
+      </c>
+      <c r="D9" t="n">
+        <v>15084.75</v>
       </c>
     </row>
   </sheetData>
@@ -796,7 +2080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -824,12 +2108,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -838,18 +2122,18 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4200.5</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -858,87 +2142,767 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>899.9</v>
+        <v>1850.45</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>23700</v>
+        <v>920.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6800</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>740.3099999999999</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4100.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1180.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>6120</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2310.1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1340.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>14850</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>servicos</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>receita</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>4600</v>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4650</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4525</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1740.55</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>860.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>vendas</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>11800</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6335.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2088.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>980.15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>vendas</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>3895</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2790</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1125.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>16300</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>8800</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6840</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2645.7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1495.35</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>17150</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>7210</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1985.25</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>10200</v>
       </c>
     </row>
   </sheetData>
@@ -974,7 +2938,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -984,7 +2948,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.29</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="4">
@@ -994,7 +2958,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5">
@@ -1004,7 +2968,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.26</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat: ampliar portfolio com narrativa consultiva e analise de receitas
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_gerencial_padronizado.xlsx
+++ b/relatorios/relatorio_gerencial_padronizado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,25 +647,25 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46058</v>
+        <v>46052</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Renovacao contratos B2B</t>
+          <t>Desconto comercial campanha janeiro</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>9100</v>
+        <v>420</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -674,25 +674,25 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>9100</v>
+        <v>-420</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46062</v>
+        <v>46058</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Treinamento corporativo</t>
+          <t>Renovacao contratos B2B</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -701,11 +701,11 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5200</v>
+        <v>9100</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>educacao</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -714,34 +714,34 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>5200</v>
+        <v>9100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46066</v>
+        <v>46062</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fornecedor homologado</t>
+          <t>Treinamento corporativo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4100.8</v>
+        <v>5200</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>educacao</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -750,21 +750,21 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>-4100.8</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46071</v>
+        <v>46066</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ferramentas analiticas</t>
+          <t>Fornecedor homologado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -773,11 +773,11 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1180.25</v>
+        <v>4100.8</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -786,21 +786,21 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>-1180.25</v>
+        <v>-4100.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46079</v>
+        <v>46071</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Comissao comercial</t>
+          <t>Ferramentas analiticas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -809,11 +809,11 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2890</v>
+        <v>1180.25</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>comercial</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -822,106 +822,106 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>-2890</v>
+        <v>-1180.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46085</v>
+        <v>46079</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Projeto de integracao beta</t>
+          <t>Comissao comercial</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>14850</v>
+        <v>2890</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>consultoria</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>14850</v>
+        <v>-2890</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46092</v>
+        <v>46080</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Receita de suporte premium</t>
+          <t>Desconto promocional fevereiro</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4650</v>
+        <v>390</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>sucesso_cliente</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>4650</v>
+        <v>-390</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46095</v>
+        <v>46085</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Campanha de retencao</t>
+          <t>Projeto de integracao beta</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2310.1</v>
+        <v>14850</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>consultoria</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -930,34 +930,34 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>-2310.1</v>
+        <v>14850</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46100</v>
+        <v>46092</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Licencas de software</t>
+          <t>Receita de suporte premium</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1340.6</v>
+        <v>4650</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>sucesso_cliente</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -966,21 +966,21 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>-1340.6</v>
+        <v>4650</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46108</v>
+        <v>46095</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Folha salarial</t>
+          <t>Campanha de retencao</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -989,11 +989,11 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>6120</v>
+        <v>2310.1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>rh</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1002,93 +1002,93 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>-6120</v>
+        <v>-2310.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46114</v>
+        <v>46100</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pacote de consultoria recorrente</t>
+          <t>Licencas de software</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>6900</v>
+        <v>1340.6</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>consultoria</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>6900</v>
+        <v>-1340.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46120</v>
+        <v>46108</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Expansao de contas enterprise</t>
+          <t>Folha salarial</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>11800</v>
+        <v>6120</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>comercial</t>
+          <t>rh</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>11800</v>
+        <v>-6120</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46127</v>
+        <v>46111</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Viagens comerciais</t>
+          <t>Desconto negociacao marco</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1740.55</v>
+        <v>430</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1106,38 +1106,38 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>-1740.55</v>
+        <v>-430</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46130</v>
+        <v>46114</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Servicos terceirizados</t>
+          <t>Pacote de consultoria recorrente</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4525</v>
+        <v>6900</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>consultoria</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1146,34 +1146,34 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>-4525</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46136</v>
+        <v>46120</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Energia e utilidades</t>
+          <t>Expansao de contas enterprise</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>vendas</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>860.9</v>
+        <v>11800</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1182,30 +1182,30 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-860.9</v>
+        <v>11800</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46148</v>
+        <v>46127</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Novos contratos SMB</t>
+          <t>Viagens comerciais</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>9700</v>
+        <v>1740.55</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1214,61 +1214,61 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>9700</v>
+        <v>-1740.55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46152</v>
+        <v>46130</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Receita de onboarding</t>
+          <t>Servicos terceirizados</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>4300</v>
+        <v>4525</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>educacao</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>4300</v>
+        <v>-4525</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46155</v>
+        <v>46136</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Eventos e comunidade</t>
+          <t>Energia e utilidades</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>infraestrutura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1277,34 +1277,34 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2088.4</v>
+        <v>860.9</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>adm</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>-2088.4</v>
+        <v>-860.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46161</v>
+        <v>46141</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Upgrade de seguranca</t>
+          <t>Desconto upgrade abril</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1313,47 +1313,47 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>980.15</v>
+        <v>410</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>-980.15</v>
+        <v>-410</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46170</v>
+        <v>46148</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Beneficios e encargos</t>
+          <t>Novos contratos SMB</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>vendas</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>6335.2</v>
+        <v>9700</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>rh</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1362,21 +1362,21 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>-6335.2</v>
+        <v>9700</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46176</v>
+        <v>46152</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Projeto analytics gamma</t>
+          <t>Receita de onboarding</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1385,70 +1385,70 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>16300</v>
+        <v>4300</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>consultoria</t>
+          <t>educacao</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>16300</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46182</v>
+        <v>46155</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Receita de renovacao anual</t>
+          <t>Eventos e comunidade</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>8800</v>
+        <v>2088.4</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>comercial</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>8800</v>
+        <v>-2088.4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46185</v>
+        <v>46161</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Parceiros estrategicos</t>
+          <t>Upgrade de seguranca</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1457,34 +1457,34 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3895</v>
+        <v>980.15</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-3895</v>
+        <v>-980.15</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46190</v>
+        <v>46170</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Monitoramento de plataforma</t>
+          <t>Beneficios e encargos</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1493,34 +1493,34 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1125.8</v>
+        <v>6335.2</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>rh</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>-1125.8</v>
+        <v>-6335.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46199</v>
+        <v>46172</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aluguel escritorio</t>
+          <t>Desconto pacote maio</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1529,29 +1529,29 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2790</v>
+        <v>395</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-2790</v>
+        <v>-395</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46210</v>
+        <v>46176</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Squad dedicado delta</t>
+          <t>Projeto analytics gamma</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>17150</v>
+        <v>16300</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1574,25 +1574,25 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>17150</v>
+        <v>16300</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46214</v>
+        <v>46182</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pacote de suporte enterprise</t>
+          <t>Receita de renovacao anual</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1601,34 +1601,34 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>5400</v>
+        <v>8800</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>sucesso_cliente</t>
+          <t>comercial</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>5400</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46218</v>
+        <v>46185</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Recrutamento especializado</t>
+          <t>Parceiros estrategicos</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1637,34 +1637,34 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>6840</v>
+        <v>3895</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>rh</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>-6840</v>
+        <v>-3895</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46224</v>
+        <v>46190</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Campanha ABM</t>
+          <t>Monitoramento de plataforma</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1673,34 +1673,34 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>2645.7</v>
+        <v>1125.8</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>-2645.7</v>
+        <v>-1125.8</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46232</v>
+        <v>46199</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automacao de backoffice</t>
+          <t>Aluguel escritorio</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>infraestrutura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1709,43 +1709,43 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1495.35</v>
+        <v>2790</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ti</t>
+          <t>adm</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>-1495.35</v>
+        <v>-2790</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46239</v>
+        <v>46202</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Renovacao base enterprise</t>
+          <t>Desconto renovacao junho</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10200</v>
+        <v>460</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1754,20 +1754,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>10200</v>
+        <v>-460</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46242</v>
+        <v>46210</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Projeto de performance epsilon</t>
+          <t>Squad dedicado delta</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>15400</v>
+        <v>17150</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1790,61 +1790,61 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>15400</v>
+        <v>17150</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46248</v>
+        <v>46214</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Operacao de campo</t>
+          <t>Pacote de suporte enterprise</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1985.25</v>
+        <v>5400</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>sucesso_cliente</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>-1985.25</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46254</v>
+        <v>46218</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Compliance e auditoria</t>
+          <t>Recrutamento especializado</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1853,56 +1853,1064 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1320</v>
+        <v>6840</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>rh</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>-1320</v>
+        <v>-6840</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Campanha ABM</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2645.7</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>-2645.7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Automacao de backoffice</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1495.35</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>-1495.35</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Desconto volume julho</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>450</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>-450</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Renovacao base enterprise</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>10200</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Projeto de performance epsilon</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>15400</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Operacao de campo</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1985.25</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>-1985.25</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Compliance e auditoria</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>-1320</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
         <v>46261</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Folha variavel e bonus</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>pessoal</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>despesa</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
         <v>7210</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>rh</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H48" t="n">
         <v>-7210</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Desconto sazonal agosto</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>470</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>-470</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Projeto de expansao zeta</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>18200</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>18200</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Pacote premium anual</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>11200</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Midia performance</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>2380</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>-2380</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Operacao de suporte</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>2140</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>-2140</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Desconto proposta setembro</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>520</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>-520</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Projeto enterprise eta</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>19400</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>19400</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Receita de sucesso do cliente</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>6100</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>sucesso_cliente</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Licencas e compliance</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>-1650</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Despesa operacional outubro</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>2260</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>-2260</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Desconto contratual outubro</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>580</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>-580</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Projeto analytics theta</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>20100</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>20100</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46337</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Renovacao carteira enterprise</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>11800</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>11800</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46343</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Folha e encargos novembro</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>7420</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>-7420</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46349</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Infraestrutura e energia</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1580</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>-1580</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46355</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Desconto black november</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>760</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>-760</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46360</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Projeto fechamento anual iota</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>22300</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>22300</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46366</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Receita adicional de servicos</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>6900</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46372</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Campanha institucional</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>2480</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>-2480</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46378</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Operacao e logistica dezembro</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>2320</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>-2320</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46385</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Desconto fechamento dezembro</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>820</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>-820</v>
       </c>
     </row>
   </sheetData>
@@ -1916,7 +2924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1948,13 +2956,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8170.75</v>
+        <v>8590.75</v>
       </c>
       <c r="C2" t="n">
         <v>21000</v>
       </c>
       <c r="D2" t="n">
-        <v>12829.25</v>
+        <v>12409.25</v>
       </c>
     </row>
     <row r="3">
@@ -1964,13 +2972,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8171.05</v>
+        <v>8561.049999999999</v>
       </c>
       <c r="C3" t="n">
         <v>14300</v>
       </c>
       <c r="D3" t="n">
-        <v>6128.95</v>
+        <v>5738.950000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1980,13 +2988,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9770.700000000001</v>
+        <v>10200.7</v>
       </c>
       <c r="C4" t="n">
         <v>19500</v>
       </c>
       <c r="D4" t="n">
-        <v>9729.299999999999</v>
+        <v>9299.299999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1996,13 +3004,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7126.45</v>
+        <v>7536.45</v>
       </c>
       <c r="C5" t="n">
         <v>18700</v>
       </c>
       <c r="D5" t="n">
-        <v>11573.55</v>
+        <v>11163.55</v>
       </c>
     </row>
     <row r="6">
@@ -2012,13 +3020,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9403.75</v>
+        <v>9798.75</v>
       </c>
       <c r="C6" t="n">
         <v>14000</v>
       </c>
       <c r="D6" t="n">
-        <v>4596.25</v>
+        <v>4201.25</v>
       </c>
     </row>
     <row r="7">
@@ -2028,13 +3036,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7810.8</v>
+        <v>8270.799999999999</v>
       </c>
       <c r="C7" t="n">
         <v>25100</v>
       </c>
       <c r="D7" t="n">
-        <v>17289.2</v>
+        <v>16829.2</v>
       </c>
     </row>
     <row r="8">
@@ -2044,13 +3052,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10981.05</v>
+        <v>11431.05</v>
       </c>
       <c r="C8" t="n">
         <v>22550</v>
       </c>
       <c r="D8" t="n">
-        <v>11568.95</v>
+        <v>11118.95</v>
       </c>
     </row>
     <row r="9">
@@ -2060,13 +3068,77 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10515.25</v>
+        <v>10985.25</v>
       </c>
       <c r="C9" t="n">
         <v>25600</v>
       </c>
       <c r="D9" t="n">
-        <v>15084.75</v>
+        <v>14614.75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5040</v>
+      </c>
+      <c r="C10" t="n">
+        <v>29400</v>
+      </c>
+      <c r="D10" t="n">
+        <v>24360</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4490</v>
+      </c>
+      <c r="C11" t="n">
+        <v>25500</v>
+      </c>
+      <c r="D11" t="n">
+        <v>21010</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>9760</v>
+      </c>
+      <c r="C12" t="n">
+        <v>31900</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22140</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5620</v>
+      </c>
+      <c r="C13" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D13" t="n">
+        <v>23580</v>
       </c>
     </row>
   </sheetData>
@@ -2080,7 +3152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2173,16 +3245,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12600</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6">
@@ -2193,7 +3265,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2202,27 +3274,27 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4100.8</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="8">
@@ -2233,7 +3305,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2242,7 +3314,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2890</v>
+        <v>4100.8</v>
       </c>
     </row>
     <row r="9">
@@ -2253,7 +3325,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2262,7 +3334,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1180.25</v>
+        <v>2890</v>
       </c>
     </row>
     <row r="10">
@@ -2273,16 +3345,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>9100</v>
+        <v>1180.25</v>
       </c>
     </row>
     <row r="11">
@@ -2293,56 +3365,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5200</v>
+        <v>390</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6120</v>
+        <v>9100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2310.1</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="14">
@@ -2353,7 +3425,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2362,7 +3434,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1340.6</v>
+        <v>6120</v>
       </c>
     </row>
     <row r="15">
@@ -2373,16 +3445,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>14850</v>
+        <v>2310.1</v>
       </c>
     </row>
     <row r="16">
@@ -2393,27 +3465,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4650</v>
+        <v>1340.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2422,47 +3494,47 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4525</v>
+        <v>430</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1740.55</v>
+        <v>14850</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>860.9</v>
+        <v>4650</v>
       </c>
     </row>
     <row r="20">
@@ -2473,16 +3545,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>11800</v>
+        <v>4525</v>
       </c>
     </row>
     <row r="21">
@@ -2493,27 +3565,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>operacoes</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6900</v>
+        <v>1740.55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>infraestrutura</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2522,18 +3594,18 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6335.2</v>
+        <v>860.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2542,38 +3614,38 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2088.4</v>
+        <v>410</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>vendas</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>980.15</v>
+        <v>11800</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vendas</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2582,7 +3654,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9700</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="26">
@@ -2593,27 +3665,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>4300</v>
+        <v>6335.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>fornecedores</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2622,18 +3694,18 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3895</v>
+        <v>2088.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2642,18 +3714,18 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2790</v>
+        <v>980.15</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tecnologia</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2662,18 +3734,18 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1125.8</v>
+        <v>395</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>vendas</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2682,18 +3754,18 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>16300</v>
+        <v>9700</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>assinaturas</t>
+          <t>servicos</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2702,18 +3774,18 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>8800</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>fornecedores</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2722,18 +3794,18 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6840</v>
+        <v>3895</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>marketing</t>
+          <t>infraestrutura</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2742,13 +3814,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2645.7</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2762,38 +3834,38 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1495.35</v>
+        <v>1125.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>descontos_comerciais</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>17150</v>
+        <v>460</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>servicos</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2802,38 +3874,38 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5400</v>
+        <v>16300</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>pessoal</t>
+          <t>assinaturas</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>despesa</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7210</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>operacoes</t>
+          <t>pessoal</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2842,18 +3914,18 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1985.25</v>
+        <v>6840</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>infraestrutura</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2862,47 +3934,607 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1320</v>
+        <v>2645.7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>tecnologia</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>receita</t>
+          <t>despesa</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>15400</v>
+        <v>1495.35</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>17150</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>7210</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1985.25</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>assinaturas</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>receita</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
         <v>10200</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>18200</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>19400</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>7420</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>20100</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>11800</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2320</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>22300</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>6900</v>
       </c>
     </row>
   </sheetData>
@@ -2938,7 +4570,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3">
@@ -2948,7 +4580,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.67</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="4">
@@ -2958,7 +4590,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="5">
@@ -2968,7 +4600,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.47</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat: ampliar base historica para novas analises
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_gerencial_padronizado.xlsx
+++ b/relatorios/relatorio_gerencial_padronizado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2910,6 +2910,1086 @@
         </is>
       </c>
       <c r="H69" t="n">
+        <v>-820</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46395</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Renovacao enterprise janeiro</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>12400</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>12400</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46400</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Projeto performance lambda</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>23100</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>23100</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46406</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Campanha digital janeiro</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>2750</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>-2750</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46411</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Operacao distribuida janeiro</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>2460</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>-2460</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46417</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Desconto comercial janeiro 2027</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>690</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>-690</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46424</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Pacote premium fevereiro</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>12900</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>12900</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46428</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Projeto transformacao mu</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>23800</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>23800</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46434</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Licencas e dados fevereiro</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1890</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>-1890</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46440</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Folha operacional fevereiro</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>7680</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>-7680</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46445</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Desconto campanha fevereiro 2027</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>710</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>-710</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46451</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Receita onboarding corporativo</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>8200</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46457</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Projeto analytics nu</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>24500</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46463</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Midia de aquisicao marco</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>2860</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>-2860</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46469</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Infraestrutura cloud marco</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1760</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>-1760</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46475</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Desconto negociacao marco 2027</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>730</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>-730</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46484</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Receita suporte premium abril</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>8600</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>sucesso_cliente</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>8600</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46489</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Projeto expansao xi</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>25200</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46495</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Compliance e auditoria abril</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1690</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>-1690</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46501</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Operacao de campo abril</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2590</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>-2590</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46506</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Desconto upgrade abril 2027</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>760</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>-760</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46513</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Renovacao carteira maio</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>13300</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>13300</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46517</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Projeto dados omicron</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>26100</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46523</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Eventos e comunidade maio</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>2980</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>-2980</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46528</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Folha e encargos maio</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>7890</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>rh</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>-7890</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46535</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Desconto promocional maio 2027</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>780</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>-780</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46542</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Receita servicos especiais junho</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>46547</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Projeto consolidacao pi</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>26800</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>26800</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46553</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Monitoramento de plataforma junho</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1980</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ti</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>-1980</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46560</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Parceiros estrategicos junho</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>4360</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>-4360</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46567</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Desconto renovacao junho 2027</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>820</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
         <v>-820</v>
       </c>
     </row>
@@ -2924,7 +4004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3139,6 +4219,102 @@
       </c>
       <c r="D13" t="n">
         <v>23580</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5900</v>
+      </c>
+      <c r="C14" t="n">
+        <v>35500</v>
+      </c>
+      <c r="D14" t="n">
+        <v>29600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10280</v>
+      </c>
+      <c r="C15" t="n">
+        <v>36700</v>
+      </c>
+      <c r="D15" t="n">
+        <v>26420</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5350</v>
+      </c>
+      <c r="C16" t="n">
+        <v>32700</v>
+      </c>
+      <c r="D16" t="n">
+        <v>27350</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5040</v>
+      </c>
+      <c r="C17" t="n">
+        <v>33800</v>
+      </c>
+      <c r="D17" t="n">
+        <v>28760</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>11650</v>
+      </c>
+      <c r="C18" t="n">
+        <v>39400</v>
+      </c>
+      <c r="D18" t="n">
+        <v>27750</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>7160</v>
+      </c>
+      <c r="C19" t="n">
+        <v>35900</v>
+      </c>
+      <c r="D19" t="n">
+        <v>28740</v>
       </c>
     </row>
   </sheetData>
@@ -3152,7 +4328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4535,6 +5711,606 @@
       </c>
       <c r="D69" t="n">
         <v>6900</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>23100</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>12400</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>7680</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1890</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>23800</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>12900</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>1760</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>24500</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>operacoes</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>2590</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>infraestrutura</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>8600</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>pessoal</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>7890</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>assinaturas</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>13300</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>fornecedores</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>4360</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>tecnologia</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>descontos_comerciais</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>projetos</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>26800</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>servicos</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>9100</v>
       </c>
     </row>
   </sheetData>
@@ -4570,7 +6346,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
@@ -4580,7 +6356,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.83</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="4">
@@ -4590,7 +6366,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.34</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="5">
@@ -4600,7 +6376,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.49</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat: adiciona analises avancadas financeiras e dashboard gerencial
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_gerencial_padronizado.xlsx
+++ b/relatorios/relatorio_gerencial_padronizado.xlsx
@@ -11,6 +11,9 @@
     <sheet name="resumo_mensal" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="resumo_categoria" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="indicadores" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="projecao" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="rentabilidade" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="liquidez" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6392,4 +6395,1243 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano_mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_receita</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>total_despesa</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>saldo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8590.75</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12409.25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>14300</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8561.049999999999</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5738.950000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>19500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10200.7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9299.299999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>18700</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7536.45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11163.55</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9798.75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4201.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>25100</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8270.799999999999</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16829.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22550</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11431.05</v>
+      </c>
+      <c r="E8" t="n">
+        <v>11118.95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>25600</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10985.25</v>
+      </c>
+      <c r="E9" t="n">
+        <v>14614.75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>29400</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5040</v>
+      </c>
+      <c r="E10" t="n">
+        <v>24360</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>25500</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4490</v>
+      </c>
+      <c r="E11" t="n">
+        <v>21010</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>31900</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9760</v>
+      </c>
+      <c r="E12" t="n">
+        <v>22140</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5620</v>
+      </c>
+      <c r="E13" t="n">
+        <v>23580</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>35500</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5900</v>
+      </c>
+      <c r="E14" t="n">
+        <v>29600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>36700</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10280</v>
+      </c>
+      <c r="E15" t="n">
+        <v>26420</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>32700</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5350</v>
+      </c>
+      <c r="E16" t="n">
+        <v>27350</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>33800</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5040</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28760</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>39400</v>
+      </c>
+      <c r="D18" t="n">
+        <v>11650</v>
+      </c>
+      <c r="E18" t="n">
+        <v>27750</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>historico</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>35900</v>
+      </c>
+      <c r="D19" t="n">
+        <v>7160</v>
+      </c>
+      <c r="E19" t="n">
+        <v>28740</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2027-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>37236.10138532019</v>
+      </c>
+      <c r="D20" t="n">
+        <v>8171.215275580646</v>
+      </c>
+      <c r="E20" t="n">
+        <v>29064.88610973954</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2027-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>36760.87138682465</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7999.660141654248</v>
+      </c>
+      <c r="E21" t="n">
+        <v>28761.2112451704</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2027-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>36929.90313392964</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8028.764887881113</v>
+      </c>
+      <c r="E22" t="n">
+        <v>28901.13824604853</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2027-10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>36869.78123165113</v>
+      </c>
+      <c r="D23" t="n">
+        <v>8023.82719681036</v>
+      </c>
+      <c r="E23" t="n">
+        <v>28845.95403484077</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2027-11</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>36891.1656354421</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8024.664888124352</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28866.50074731775</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2027-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>projecao</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>36883.55954334979</v>
+      </c>
+      <c r="D25" t="n">
+        <v>8024.52277175306</v>
+      </c>
+      <c r="E25" t="n">
+        <v>28859.03677159673</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>centro_custo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>total_receita</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_despesa</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>peso_receita</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>despesa_alocada_suporte</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>despesa_total_alocada</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>margem_liquida</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>margem_percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>consultoria</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>312700</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.6371879775853285</v>
+      </c>
+      <c r="E2" t="n">
+        <v>45914.84174223128</v>
+      </c>
+      <c r="F2" t="n">
+        <v>45914.84174223128</v>
+      </c>
+      <c r="G2" t="n">
+        <v>266785.1582577687</v>
+      </c>
+      <c r="H2" t="n">
+        <v>85.31664798777382</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>comercial</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>119600</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15225.55</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2437086092715232</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17561.28900662252</v>
+      </c>
+      <c r="F3" t="n">
+        <v>32786.83900662252</v>
+      </c>
+      <c r="G3" t="n">
+        <v>86813.16099337747</v>
+      </c>
+      <c r="H3" t="n">
+        <v>72.58625501118517</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>educacao</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>33700</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.06867040244523688</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4948.289628120224</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4948.289628120224</v>
+      </c>
+      <c r="G4" t="n">
+        <v>28751.71037187978</v>
+      </c>
+      <c r="H4" t="n">
+        <v>85.31664798777382</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sucesso_cliente</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24750</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.05043301069791136</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3634.129623025981</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3634.129623025981</v>
+      </c>
+      <c r="G5" t="n">
+        <v>21115.87037697402</v>
+      </c>
+      <c r="H5" t="n">
+        <v>85.31664798777382</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano_mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>saidas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>entradas</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>saldo_caixa</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>saldo_acumulado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ciclo_caixa_dias</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>necessidade_capital_giro</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7670.45</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8400</v>
+      </c>
+      <c r="D2" t="n">
+        <v>729.5500000000002</v>
+      </c>
+      <c r="E2" t="n">
+        <v>729.5500000000002</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4200.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>21700</v>
+      </c>
+      <c r="D3" t="n">
+        <v>17499.7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>18229.25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14141.15</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9850</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-4291.15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>13938.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1750.6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>21750</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19999.4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>33937.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15945.05</v>
+      </c>
+      <c r="C6" t="n">
+        <v>25800</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9854.950000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>43792.45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1440.15</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8800</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7359.85</v>
+      </c>
+      <c r="E7" t="n">
+        <v>51152.3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15100.8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>21700</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6599.200000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>57751.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>13141.05</v>
+      </c>
+      <c r="C9" t="n">
+        <v>27350</v>
+      </c>
+      <c r="D9" t="n">
+        <v>14208.95</v>
+      </c>
+      <c r="E9" t="n">
+        <v>71960.45</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2505.25</v>
+      </c>
+      <c r="C10" t="n">
+        <v>26600</v>
+      </c>
+      <c r="D10" t="n">
+        <v>24094.75</v>
+      </c>
+      <c r="E10" t="n">
+        <v>96055.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="C11" t="n">
+        <v>18200</v>
+      </c>
+      <c r="D11" t="n">
+        <v>13100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>109155.2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>12090</v>
+      </c>
+      <c r="C12" t="n">
+        <v>37300</v>
+      </c>
+      <c r="D12" t="n">
+        <v>25210</v>
+      </c>
+      <c r="E12" t="n">
+        <v>134365.2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4880</v>
+      </c>
+      <c r="C13" t="n">
+        <v>27000</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22120</v>
+      </c>
+      <c r="E13" t="n">
+        <v>156485.2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3010</v>
+      </c>
+      <c r="C14" t="n">
+        <v>34700</v>
+      </c>
+      <c r="D14" t="n">
+        <v>31690</v>
+      </c>
+      <c r="E14" t="n">
+        <v>188175.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>13600</v>
+      </c>
+      <c r="C15" t="n">
+        <v>36000</v>
+      </c>
+      <c r="D15" t="n">
+        <v>22400</v>
+      </c>
+      <c r="E15" t="n">
+        <v>210575.2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2620</v>
+      </c>
+      <c r="C16" t="n">
+        <v>32000</v>
+      </c>
+      <c r="D16" t="n">
+        <v>29380</v>
+      </c>
+      <c r="E16" t="n">
+        <v>239955.2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7070</v>
+      </c>
+      <c r="C17" t="n">
+        <v>33100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>26030</v>
+      </c>
+      <c r="E17" t="n">
+        <v>265985.2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>14240</v>
+      </c>
+      <c r="C18" t="n">
+        <v>38500</v>
+      </c>
+      <c r="D18" t="n">
+        <v>24260</v>
+      </c>
+      <c r="E18" t="n">
+        <v>290245.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>820</v>
+      </c>
+      <c r="C19" t="n">
+        <v>35200</v>
+      </c>
+      <c r="D19" t="n">
+        <v>34380</v>
+      </c>
+      <c r="E19" t="n">
+        <v>324625.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2027-07</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6340</v>
+      </c>
+      <c r="C20" t="n">
+        <v>26800</v>
+      </c>
+      <c r="D20" t="n">
+        <v>20460</v>
+      </c>
+      <c r="E20" t="n">
+        <v>345085.2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>